<commit_message>
Water meters replaced, elec AMR installed unit 63
</commit_message>
<xml_diff>
--- a/EVG_SIT_FS_Meter_Commissioning_2026-07-01.xlsx
+++ b/EVG_SIT_FS_Meter_Commissioning_2026-07-01.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://voltano-my.sharepoint.com/personal/ruan_vh_voltano_com/Documents/Desktop/Voltano/Clients/Evergreen/Evergreen Sitari/Site initialization/Freestanding/EVG_FS_Project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4277" documentId="8_{C97FC332-2E41-401D-B97C-40A4EC775E62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A8BA02EC-B27E-4DAB-8A4A-7A36ABB01727}"/>
+  <xr:revisionPtr revIDLastSave="4314" documentId="8_{C97FC332-2E41-401D-B97C-40A4EC775E62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A21BD7F9-D0A2-4495-AD3E-7444FDE1190E}"/>
   <bookViews>
-    <workbookView xWindow="59280" yWindow="-2430" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FS Elec" sheetId="4" r:id="rId1"/>
@@ -26,7 +26,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'FS Elec'!$A$1:$U$192</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'FS Water'!$A$1:$T$193</definedName>
   </definedNames>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="191028" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5123" uniqueCount="1332">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5128" uniqueCount="1333">
   <si>
     <t xml:space="preserve">Stand Number </t>
   </si>
@@ -4043,6 +4043,9 @@
   </si>
   <si>
     <t>54789022</t>
+  </si>
+  <si>
+    <t>probe removed</t>
   </si>
 </sst>
 </file>
@@ -4710,7 +4713,7 @@
     <xf numFmtId="0" fontId="20" fillId="37" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="160">
+  <cellXfs count="162">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -5184,16 +5187,22 @@
     <xf numFmtId="14" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -5203,7 +5212,87 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="3" xr:uid="{0A8ABF22-C885-4E8B-8CEC-181E323DF71D}"/>
   </cellStyles>
-  <dxfs count="35">
+  <dxfs count="43">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -5896,7 +5985,7 @@
     <col min="11" max="11" width="27.265625" style="5" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="16.59765625" customWidth="1"/>
     <col min="13" max="13" width="18.3984375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.3984375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="13.1328125" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="17.3984375" bestFit="1" customWidth="1"/>
     <col min="16" max="19" width="11.265625" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="16.86328125" bestFit="1" customWidth="1"/>
@@ -7317,7 +7406,7 @@
       <c r="B24" s="29" t="s">
         <v>27</v>
       </c>
-      <c r="C24" s="158">
+      <c r="C24" s="156">
         <v>14558068921</v>
       </c>
       <c r="D24" s="2">
@@ -9730,7 +9819,7 @@
         <v>1286</v>
       </c>
       <c r="N63" s="2">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="O63" s="64" t="s">
         <v>130</v>
@@ -9785,12 +9874,12 @@
         <v>46197</v>
       </c>
       <c r="L64" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M64" s="2" t="s">
         <v>1286</v>
       </c>
-      <c r="N64" s="7">
+      <c r="N64" s="159">
         <v>2</v>
       </c>
       <c r="O64" s="64" t="s">
@@ -10940,7 +11029,7 @@
       <c r="B83" s="26" t="s">
         <v>65</v>
       </c>
-      <c r="C83" s="158">
+      <c r="C83" s="156">
         <v>14558069077</v>
       </c>
       <c r="D83" s="2">
@@ -13850,7 +13939,7 @@
       <c r="M128" s="2" t="s">
         <v>1214</v>
       </c>
-      <c r="N128" s="159">
+      <c r="N128" s="2">
         <v>7</v>
       </c>
       <c r="O128" s="64" t="s">
@@ -14098,7 +14187,7 @@
       <c r="M132" s="2" t="s">
         <v>1214</v>
       </c>
-      <c r="N132" s="159">
+      <c r="N132" s="2">
         <v>1</v>
       </c>
       <c r="O132" s="64" t="s">
@@ -15347,8 +15436,8 @@
       <c r="M153" s="2" t="s">
         <v>1288</v>
       </c>
-      <c r="N153" s="7">
-        <v>8</v>
+      <c r="N153" s="7" t="s">
+        <v>1332</v>
       </c>
       <c r="O153" s="64" t="s">
         <v>37</v>
@@ -15652,7 +15741,7 @@
       <c r="M158" s="2" t="s">
         <v>1287</v>
       </c>
-      <c r="N158" s="159">
+      <c r="N158" s="2">
         <v>2</v>
       </c>
       <c r="O158" s="64" t="s">
@@ -15713,7 +15802,7 @@
       <c r="M159" s="2" t="s">
         <v>1287</v>
       </c>
-      <c r="N159" s="159">
+      <c r="N159" s="2">
         <v>3</v>
       </c>
       <c r="O159" s="64" t="s">
@@ -15774,7 +15863,7 @@
       <c r="M160" s="2" t="s">
         <v>1287</v>
       </c>
-      <c r="N160" s="159">
+      <c r="N160" s="2">
         <v>8</v>
       </c>
       <c r="O160" s="64" t="s">
@@ -15835,7 +15924,7 @@
       <c r="M161" s="2" t="s">
         <v>1287</v>
       </c>
-      <c r="N161" s="159">
+      <c r="N161" s="2">
         <v>4</v>
       </c>
       <c r="O161" s="64" t="s">
@@ -15896,7 +15985,7 @@
       <c r="M162" s="2" t="s">
         <v>1287</v>
       </c>
-      <c r="N162" s="159">
+      <c r="N162" s="2">
         <v>5</v>
       </c>
       <c r="O162" s="64" t="s">
@@ -15957,7 +16046,7 @@
       <c r="M163" s="2" t="s">
         <v>1287</v>
       </c>
-      <c r="N163" s="159">
+      <c r="N163" s="2">
         <v>6</v>
       </c>
       <c r="O163" s="64" t="s">
@@ -16018,7 +16107,7 @@
       <c r="M164" s="2" t="s">
         <v>1281</v>
       </c>
-      <c r="N164" s="159">
+      <c r="N164" s="2">
         <v>6</v>
       </c>
       <c r="O164" s="64" t="s">
@@ -16079,7 +16168,7 @@
       <c r="M165" s="2" t="s">
         <v>1281</v>
       </c>
-      <c r="N165" s="159">
+      <c r="N165" s="2">
         <v>3</v>
       </c>
       <c r="O165" s="64" t="s">
@@ -16140,7 +16229,7 @@
       <c r="M166" s="2" t="s">
         <v>1281</v>
       </c>
-      <c r="N166" s="159">
+      <c r="N166" s="2">
         <v>2</v>
       </c>
       <c r="O166" s="64" t="s">
@@ -16201,7 +16290,7 @@
       <c r="M167" s="2" t="s">
         <v>1281</v>
       </c>
-      <c r="N167" s="159">
+      <c r="N167" s="2">
         <v>1</v>
       </c>
       <c r="O167" s="64" t="s">
@@ -16262,7 +16351,7 @@
       <c r="M168" s="2" t="s">
         <v>1281</v>
       </c>
-      <c r="N168" s="159">
+      <c r="N168" s="2">
         <v>5</v>
       </c>
       <c r="O168" s="64" t="s">
@@ -16323,7 +16412,7 @@
       <c r="M169" s="2" t="s">
         <v>1281</v>
       </c>
-      <c r="N169" s="159">
+      <c r="N169" s="2">
         <v>7</v>
       </c>
       <c r="O169" s="64" t="s">
@@ -16384,7 +16473,7 @@
       <c r="M170" s="2" t="s">
         <v>1281</v>
       </c>
-      <c r="N170" s="159">
+      <c r="N170" s="2">
         <v>4</v>
       </c>
       <c r="O170" s="64" t="s">
@@ -16445,7 +16534,7 @@
       <c r="M171" s="2" t="s">
         <v>1226</v>
       </c>
-      <c r="N171" s="159">
+      <c r="N171" s="2">
         <v>1</v>
       </c>
       <c r="O171" s="64" t="s">
@@ -16506,7 +16595,7 @@
       <c r="M172" s="2" t="s">
         <v>1226</v>
       </c>
-      <c r="N172" s="159">
+      <c r="N172" s="2">
         <v>2</v>
       </c>
       <c r="O172" s="64" t="s">
@@ -16567,7 +16656,7 @@
       <c r="M173" s="2" t="s">
         <v>1226</v>
       </c>
-      <c r="N173" s="159">
+      <c r="N173" s="2">
         <v>3</v>
       </c>
       <c r="O173" s="64" t="s">
@@ -16628,7 +16717,7 @@
       <c r="M174" s="2" t="s">
         <v>1226</v>
       </c>
-      <c r="N174" s="159">
+      <c r="N174" s="2">
         <v>4</v>
       </c>
       <c r="O174" s="64" t="s">
@@ -16689,7 +16778,7 @@
       <c r="M175" s="2" t="s">
         <v>1226</v>
       </c>
-      <c r="N175" s="159">
+      <c r="N175" s="2">
         <v>5</v>
       </c>
       <c r="O175" s="64" t="s">
@@ -16750,7 +16839,7 @@
       <c r="M176" s="2" t="s">
         <v>1226</v>
       </c>
-      <c r="N176" s="159">
+      <c r="N176" s="2">
         <v>6</v>
       </c>
       <c r="O176" s="64" t="s">
@@ -16811,7 +16900,7 @@
       <c r="M177" s="2" t="s">
         <v>1225</v>
       </c>
-      <c r="N177" s="159">
+      <c r="N177" s="2">
         <v>1</v>
       </c>
       <c r="O177" s="64" t="s">
@@ -17753,13 +17842,13 @@
   </sortState>
   <phoneticPr fontId="11" type="noConversion"/>
   <conditionalFormatting sqref="C25:C192 C2:C23">
-    <cfRule type="duplicateValues" dxfId="34" priority="8"/>
+    <cfRule type="duplicateValues" dxfId="42" priority="8"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C117:C122">
-    <cfRule type="duplicateValues" dxfId="33" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="41" priority="3"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C124:C132">
-    <cfRule type="duplicateValues" dxfId="32" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="40" priority="2"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -21043,8 +21132,8 @@
       <c r="B62" s="60" t="s">
         <v>27</v>
       </c>
-      <c r="C62" s="53" t="s">
-        <v>314</v>
+      <c r="C62" s="160">
+        <v>10852211</v>
       </c>
       <c r="D62" s="53" t="s">
         <v>284</v>
@@ -21062,7 +21151,7 @@
         <v>46186</v>
       </c>
       <c r="I62" s="21" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J62" s="63" t="s">
         <v>132</v>
@@ -21080,12 +21169,14 @@
         <v>46179</v>
       </c>
       <c r="O62" s="21" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P62" s="21" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q62" s="17"/>
+        <v>1</v>
+      </c>
+      <c r="Q62" s="57">
+        <v>46318</v>
+      </c>
       <c r="R62" s="136"/>
       <c r="S62" s="136"/>
     </row>
@@ -21471,8 +21562,8 @@
       <c r="B70" s="60" t="s">
         <v>27</v>
       </c>
-      <c r="C70" s="53" t="s">
-        <v>320</v>
+      <c r="C70" s="160">
+        <v>10852373</v>
       </c>
       <c r="D70" s="53" t="s">
         <v>284</v>
@@ -21490,7 +21581,7 @@
         <v>46186</v>
       </c>
       <c r="I70" s="21" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J70" s="63" t="s">
         <v>132</v>
@@ -21508,12 +21599,14 @@
         <v>46179</v>
       </c>
       <c r="O70" s="21" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P70" s="21" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q70" s="17"/>
+        <v>1</v>
+      </c>
+      <c r="Q70" s="57">
+        <v>46318</v>
+      </c>
       <c r="R70" s="136"/>
       <c r="S70" s="136"/>
     </row>
@@ -28059,11 +28152,11 @@
     <sortCondition ref="A2:A193"/>
   </sortState>
   <phoneticPr fontId="11" type="noConversion"/>
-  <conditionalFormatting sqref="C2:C3 C5:C63">
-    <cfRule type="duplicateValues" dxfId="31" priority="2"/>
-    <cfRule type="duplicateValues" dxfId="30" priority="5"/>
-    <cfRule type="duplicateValues" dxfId="29" priority="6"/>
-    <cfRule type="duplicateValues" dxfId="28" priority="7"/>
+  <conditionalFormatting sqref="C2:C3 C5:C61 C63">
+    <cfRule type="duplicateValues" dxfId="39" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="38" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="37" priority="10"/>
+    <cfRule type="duplicateValues" dxfId="36" priority="11"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -33785,7 +33878,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="C143:C268">
-    <cfRule type="duplicateValues" dxfId="27" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="35" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -38072,22 +38165,22 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="C2:D125">
-    <cfRule type="duplicateValues" dxfId="26" priority="6" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="34" priority="6" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C126:D251">
-    <cfRule type="duplicateValues" dxfId="25" priority="5" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="33" priority="5" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E126:E251">
-    <cfRule type="cellIs" dxfId="24" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="32" priority="1" operator="equal">
       <formula>"In Progress"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="23" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="31" priority="2" operator="equal">
       <formula>"Maybe"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="22" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="30" priority="3" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="21" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="29" priority="4" operator="equal">
       <formula>"No"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -38112,34 +38205,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="14.65" x14ac:dyDescent="0.45">
-      <c r="A1" s="156" t="s">
+      <c r="A1" s="157" t="s">
         <v>1164</v>
       </c>
-      <c r="B1" s="156" t="s">
+      <c r="B1" s="157" t="s">
         <v>1165</v>
       </c>
-      <c r="C1" s="156" t="s">
+      <c r="C1" s="157" t="s">
         <v>1166</v>
       </c>
-      <c r="D1" s="157" t="s">
+      <c r="D1" s="158" t="s">
         <v>1167</v>
       </c>
-      <c r="E1" s="157"/>
-      <c r="F1" s="157"/>
-      <c r="G1" s="157" t="s">
+      <c r="E1" s="158"/>
+      <c r="F1" s="158"/>
+      <c r="G1" s="158" t="s">
         <v>1168</v>
       </c>
-      <c r="H1" s="157"/>
-      <c r="I1" s="157"/>
+      <c r="H1" s="158"/>
+      <c r="I1" s="158"/>
       <c r="J1" s="108"/>
       <c r="K1" s="109" t="s">
         <v>1169</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="14.65" x14ac:dyDescent="0.45">
-      <c r="A2" s="156"/>
-      <c r="B2" s="156"/>
-      <c r="C2" s="156"/>
+      <c r="A2" s="157"/>
+      <c r="B2" s="157"/>
+      <c r="C2" s="157"/>
       <c r="D2" s="107" t="s">
         <v>1170</v>
       </c>
@@ -40642,7 +40735,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E8F51D9-DC2A-407D-9B2E-297FBBC4C6A6}">
-  <dimension ref="A1:I24"/>
+  <dimension ref="A1:I26"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17" bestFit="1" customWidth="1"/>
@@ -41352,42 +41445,106 @@
         <v>9.5000000000000001E-2</v>
       </c>
     </row>
+    <row r="25" spans="1:9" ht="18" x14ac:dyDescent="0.55000000000000004">
+      <c r="A25" s="23" t="s">
+        <v>164</v>
+      </c>
+      <c r="B25" s="53" t="s">
+        <v>314</v>
+      </c>
+      <c r="C25" s="53" t="s">
+        <v>285</v>
+      </c>
+      <c r="D25" s="3">
+        <v>6.7000000000000004E-2</v>
+      </c>
+      <c r="E25" s="57">
+        <v>46186</v>
+      </c>
+      <c r="F25" s="150" t="b">
+        <v>1</v>
+      </c>
+      <c r="G25" s="57">
+        <v>46318</v>
+      </c>
+      <c r="H25" s="160">
+        <v>10852211</v>
+      </c>
+      <c r="I25" s="161">
+        <v>0.106</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" ht="18" x14ac:dyDescent="0.55000000000000004">
+      <c r="A26" s="23" t="s">
+        <v>131</v>
+      </c>
+      <c r="B26" s="53" t="s">
+        <v>320</v>
+      </c>
+      <c r="C26" s="53" t="s">
+        <v>285</v>
+      </c>
+      <c r="D26" s="3">
+        <v>6.6000000000000003E-2</v>
+      </c>
+      <c r="E26" s="57">
+        <v>46186</v>
+      </c>
+      <c r="F26" s="150" t="b">
+        <v>1</v>
+      </c>
+      <c r="G26" s="57">
+        <v>46318</v>
+      </c>
+      <c r="H26" s="160">
+        <v>10852373</v>
+      </c>
+      <c r="I26" s="161">
+        <v>8.5000000000000006E-2</v>
+      </c>
+    </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I15">
     <sortCondition ref="G2:G15"/>
   </sortState>
   <conditionalFormatting sqref="A2:A16 A19:A22 A24">
-    <cfRule type="duplicateValues" dxfId="20" priority="25"/>
+    <cfRule type="duplicateValues" dxfId="28" priority="29"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B20">
-    <cfRule type="duplicateValues" dxfId="19" priority="13"/>
-    <cfRule type="duplicateValues" dxfId="18" priority="14"/>
-    <cfRule type="duplicateValues" dxfId="17" priority="15"/>
-    <cfRule type="duplicateValues" dxfId="16" priority="16"/>
+    <cfRule type="duplicateValues" dxfId="27" priority="17"/>
+    <cfRule type="duplicateValues" dxfId="26" priority="18"/>
+    <cfRule type="duplicateValues" dxfId="25" priority="19"/>
+    <cfRule type="duplicateValues" dxfId="24" priority="20"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B21">
-    <cfRule type="duplicateValues" dxfId="15" priority="9"/>
-    <cfRule type="duplicateValues" dxfId="14" priority="10"/>
-    <cfRule type="duplicateValues" dxfId="13" priority="11"/>
-    <cfRule type="duplicateValues" dxfId="12" priority="12"/>
+    <cfRule type="duplicateValues" dxfId="23" priority="13"/>
+    <cfRule type="duplicateValues" dxfId="22" priority="14"/>
+    <cfRule type="duplicateValues" dxfId="21" priority="15"/>
+    <cfRule type="duplicateValues" dxfId="20" priority="16"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B22">
-    <cfRule type="duplicateValues" dxfId="11" priority="5"/>
-    <cfRule type="duplicateValues" dxfId="10" priority="6"/>
-    <cfRule type="duplicateValues" dxfId="9" priority="7"/>
-    <cfRule type="duplicateValues" dxfId="8" priority="8"/>
+    <cfRule type="duplicateValues" dxfId="19" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="18" priority="10"/>
+    <cfRule type="duplicateValues" dxfId="17" priority="11"/>
+    <cfRule type="duplicateValues" dxfId="16" priority="12"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B24">
+    <cfRule type="duplicateValues" dxfId="15" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="14" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="13" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="12" priority="8"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H2">
+    <cfRule type="duplicateValues" dxfId="11" priority="22"/>
+    <cfRule type="duplicateValues" dxfId="10" priority="23"/>
+    <cfRule type="duplicateValues" dxfId="9" priority="24"/>
+    <cfRule type="duplicateValues" dxfId="8" priority="25"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B25">
     <cfRule type="duplicateValues" dxfId="7" priority="1"/>
     <cfRule type="duplicateValues" dxfId="6" priority="2"/>
     <cfRule type="duplicateValues" dxfId="5" priority="3"/>
     <cfRule type="duplicateValues" dxfId="4" priority="4"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H2">
-    <cfRule type="duplicateValues" dxfId="3" priority="18"/>
-    <cfRule type="duplicateValues" dxfId="2" priority="19"/>
-    <cfRule type="duplicateValues" dxfId="1" priority="20"/>
-    <cfRule type="duplicateValues" dxfId="0" priority="21"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>